<commit_message>
fix(riders): correct training-status header label in excel template
템플릿 헤더가 '(완료/미완료)'로 표기돼 손-입력 시 파서(온라인/오프라인/미완료)와
불일치하던 것을 '(온라인/오프라인/미완료)'로 정정. 샘플 셀 완료→온라인.
드롭다운은 이미 3값이라 무변경.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/development/service-ops-api/src/main/resources/templates/excel/riders-template.xlsx
+++ b/development/service-ops-api/src/main/resources/templates/excel/riders-template.xlsx
@@ -529,7 +529,7 @@
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>교육이수 *
-(완료 / 미완료)</t>
+(온라인 / 오프라인 / 미완료)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>온라인</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>온라인</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">

</xml_diff>